<commit_message>
major changes to ui
</commit_message>
<xml_diff>
--- a/src/data/coupons.xlsx
+++ b/src/data/coupons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gala\Documents\code\jk3\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DEA88E-0340-45BA-BDFB-010BE739BB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD336BE2-7C4D-45D4-947D-9624168E1BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="1236" windowWidth="11808" windowHeight="11076" xr2:uid="{6540F3E8-6E2B-46EF-8B33-43A96A14636B}"/>
+    <workbookView xWindow="8940" yWindow="924" windowWidth="12996" windowHeight="11076" xr2:uid="{6540F3E8-6E2B-46EF-8B33-43A96A14636B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,9 +74,6 @@
     <t>brand</t>
   </si>
   <si>
-    <t>Nike, Puma</t>
-  </si>
-  <si>
     <t>active</t>
   </si>
   <si>
@@ -98,10 +95,13 @@
     <t>category</t>
   </si>
   <si>
-    <t>Footwear</t>
-  </si>
-  <si>
     <t>expiryDate</t>
+  </si>
+  <si>
+    <t>Eastman, JRSDrive</t>
+  </si>
+  <si>
+    <t>Foxcare</t>
   </si>
 </sst>
 </file>
@@ -557,7 +557,7 @@
         <v>7</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>0</v>
@@ -577,7 +577,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F2" s="4">
         <v>0</v>
@@ -589,39 +589,41 @@
         <v>46265</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15" thickBot="1">
       <c r="A3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="C3" s="4">
         <v>50</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="F3" s="4">
         <v>200</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="4">
+        <v>50</v>
+      </c>
       <c r="H3" s="5">
         <v>46387</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15" thickBot="1">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>9</v>
@@ -630,10 +632,10 @@
         <v>10</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="4">
         <v>30</v>
@@ -645,7 +647,7 @@
         <v>46280</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9">

</xml_diff>